<commit_message>
Vocabulary V2: modality-group label renames + emitter source fix
Renames four modality-group display labels (group_name) to the target
state in Vocabulary_TargetState_and_Plan_v1 §3:
  foot         Foot (run / hike / nav)   -> Foot
  snow_travel  Snow travel (foot)        -> Snow Travel (on foot)
  snow_glide   Snow travel (gliding)     -> Skiing
  climb        Climbing (rope-protected) -> Roped climbing

Also corrects a V1-leftover staleness in the bike_offroad description
('Gravel folds in once D-006 splits' -> now reflects gravel/cross-country
as live members) and fixes emit_sql.py to derive the '-- Source:' header
from run.SPORTS_XLSX (was hardcoded to the stale v12 workbook name).

Re-emitted as layer0_etl_v1.6.1.sql (etl_version 0A-v1.6.1). Description-
only patch on top of the applied v1.6.0; needs a Neon apply.

https://claude.ai/code/session_019MRyhMiWEaHivR4ifueqwN
</commit_message>
<xml_diff>
--- a/etl/sources/Sports_Framework_v14.xlsx
+++ b/etl/sources/Sports_Framework_v14.xlsx
@@ -5723,7 +5723,7 @@
       </c>
       <c r="B4" s="190" t="inlineStr">
         <is>
-          <t>Foot (run / hike / nav)</t>
+          <t>Foot</t>
         </is>
       </c>
       <c r="C4" s="190" t="inlineStr">
@@ -5777,7 +5777,7 @@
       </c>
       <c r="D6" s="190" t="inlineStr">
         <is>
-          <t>Cycling disciplines on technical trail / mountain surfaces (mountain biking). Gravel folds in once D-006 splits.</t>
+          <t>Cycling disciplines on technical trail / mountain surfaces (mountain biking, gravel, cross-country).</t>
         </is>
       </c>
     </row>
@@ -5789,7 +5789,7 @@
       </c>
       <c r="B7" s="190" t="inlineStr">
         <is>
-          <t>Snow travel (foot)</t>
+          <t>Snow Travel (on foot)</t>
         </is>
       </c>
       <c r="C7" s="190" t="inlineStr">
@@ -5811,7 +5811,7 @@
       </c>
       <c r="B8" s="190" t="inlineStr">
         <is>
-          <t>Snow travel (gliding)</t>
+          <t>Skiing</t>
         </is>
       </c>
       <c r="C8" s="190" t="inlineStr">
@@ -5833,7 +5833,7 @@
       </c>
       <c r="B9" s="190" t="inlineStr">
         <is>
-          <t>Climbing (rope-protected)</t>
+          <t>Roped climbing</t>
         </is>
       </c>
       <c r="C9" s="190" t="inlineStr">
@@ -6263,85 +6263,85 @@
       <c r="C27" s="190" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="190" t="inlineStr">
         <is>
           <t>D-030</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="190" t="inlineStr">
         <is>
           <t>bike_pavement</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="190" t="inlineStr">
         <is>
           <t>Gravel cycling pools with road training</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="190" t="inlineStr">
         <is>
           <t>D-030</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="190" t="inlineStr">
         <is>
           <t>bike_offroad</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="190" t="inlineStr">
         <is>
           <t>Gravel cycling also pools with off-road training</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="190" t="inlineStr">
         <is>
           <t>D-031</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="190" t="inlineStr">
         <is>
           <t>bike_offroad</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="190" t="inlineStr">
         <is>
           <t>Cross country (XC) mountain biking</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="190" t="inlineStr">
         <is>
           <t>D-032</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="190" t="inlineStr">
         <is>
           <t>paddle_flatwater</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="190" t="inlineStr">
         <is>
           <t>Stand-up paddleboard, flatwater modality</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="190" t="inlineStr">
         <is>
           <t>D-019</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="190" t="inlineStr">
         <is>
           <t>paddle_whitewater</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="190" t="inlineStr">
         <is>
           <t>Paddle rafting on moving/whitewater</t>
         </is>
@@ -8881,201 +8881,201 @@
       </c>
     </row>
     <row r="31" ht="139.5" customHeight="1" s="191">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="190" t="inlineStr">
         <is>
           <t>D-030</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="190" t="inlineStr">
         <is>
           <t>Gravel Cycling</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="190" t="inlineStr">
         <is>
           <t>Cycling</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="190" t="inlineStr">
         <is>
           <t>Long Distance / Endurance Cycling · Adventure Racing</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E31" s="190" t="inlineStr">
         <is>
           <t>Same as Road Cycling (D-006): 2–3 weeks Zone 2 before structured intervals. Add loose-surface bike handling at low tire pressure.</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F31" s="190" t="inlineStr">
         <is>
           <t>Same structure as Road Cycling (D-006). Gravel-specific: sustained tempo on mixed surface; loose-surface handling and longer unsupported efforts in Build.</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G31" s="190" t="inlineStr">
         <is>
           <t>Same as Road Cycling (D-006): 10–15%/week ride hours; FTP intervals +1 rep or +5% duration per 2-week block, not both.</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="H31" s="190" t="inlineStr">
         <is>
           <t>Same as Road Cycling (D-006) by age group; watch patellar tendon.</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="I31" s="190" t="inlineStr">
         <is>
           <t>1–2 weeks. Volume cut 40–50%. Maintain 2 shorter intensity sessions.</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="J31" s="190" t="inlineStr">
         <is>
           <t>Knee pain (patellar tendon, IT band) · Lower back (aero position) · Hand/wrist fatigue from sustained surface vibration</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr">
+      <c r="K31" s="190" t="inlineStr">
         <is>
           <t>Rapid intensity escalation without aerobic base · Poor saddle height · Poor cleat alignment</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr">
+      <c r="L31" s="190" t="inlineStr">
         <is>
           <t>Same as Road Cycling (D-006): active recovery spin, hip flexor stretch, sleep.</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr">
+      <c r="M31" s="190" t="inlineStr">
         <is>
           <t>Gravel-specific: extrapolated from road cycling literature (Strong for the shared road-cycling claims).</t>
         </is>
       </c>
     </row>
     <row r="32" ht="139.5" customHeight="1" s="191">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="190" t="inlineStr">
         <is>
           <t>D-031</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="190" t="inlineStr">
         <is>
           <t>Cross Country Cycling</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="190" t="inlineStr">
         <is>
           <t>Cycling</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="190" t="inlineStr">
         <is>
           <t>Long Distance / Endurance Cycling · Adventure Racing · XC MTB</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E32" s="190" t="inlineStr">
         <is>
           <t>Same as Mountain Biking (D-008): 4–6 weeks road/easy-trail aerobic base and pedaling mechanics before technical XC riding.</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F32" s="190" t="inlineStr">
         <is>
           <t>Same structure as Mountain Biking (D-008), XC-racing focus: aerobic base + sustained climbing power; less technical-descent emphasis than Enduro.</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="G32" s="190" t="inlineStr">
         <is>
           <t>Same as Mountain Biking (D-008): 10–15%/week ride hours; add one new technical element per 2-week block (not by volume).</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="H32" s="190" t="inlineStr">
         <is>
           <t>Same as Mountain Biking (D-008) by age group; CNS-fatigue caps on hard technical days.</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="I32" s="190" t="inlineStr">
         <is>
           <t>1–2 weeks. Volume cut 35–50%. Maintain 1 technical skills session.</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="J32" s="190" t="inlineStr">
         <is>
           <t>Lower back pain · Knee pain (fit) · Hand/wrist numbness · Shoulder impingement · Crashes</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
+      <c r="K32" s="190" t="inlineStr">
         <is>
           <t>Skipping road base phase · Riding technically while fatigued · Poor bike fit · Insufficient core strength</t>
         </is>
       </c>
-      <c r="L32" t="inlineStr">
+      <c r="L32" s="190" t="inlineStr">
         <is>
           <t>Same as Mountain Biking (D-008): thoracic/lat foam roll, sleep, hip flexor stretch.</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr">
+      <c r="M32" s="190" t="inlineStr">
         <is>
           <t>XC-specific: shares Mountain Biking evidence base (practitioner consensus for skill/CNS).</t>
         </is>
       </c>
     </row>
     <row r="33" ht="139.5" customHeight="1" s="191">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="190" t="inlineStr">
         <is>
           <t>D-032</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="190" t="inlineStr">
         <is>
           <t>Stand-up Paddleboard</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="190" t="inlineStr">
         <is>
           <t>Water / Paddle</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="190" t="inlineStr">
         <is>
           <t>Flatwater / Touring · Adventure Racing (minor)</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E33" s="190" t="inlineStr">
         <is>
           <t>Same as Kayaking (D-010): 4–6 weeks flat-water paddle technique base. SUP-specific: build standing balance and anti-rotation core before volume.</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F33" s="190" t="inlineStr">
         <is>
           <t>Same structure as Kayaking (D-010): BASE flat-water technique + balance; BUILD volume; PEAK race-sim. Standing balance and core stability are the SUP-specific demand.</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="G33" s="190" t="inlineStr">
         <is>
           <t>Same as Kayaking (D-010): 10–15%/week paddle hours; grip sessions max 3×/week.</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="H33" s="190" t="inlineStr">
         <is>
           <t>Same as Kayaking (D-010) by age group; shoulder recovery 48–72 hr for masters.</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="I33" s="190" t="inlineStr">
         <is>
           <t>1–2 weeks. Volume cut 40–50%.</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="J33" s="190" t="inlineStr">
         <is>
           <t>Shoulder impingement / rotator cuff · Wrist tendinopathy (paddle grip) · Lower back (standing posture, anti-rotation load)</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr">
+      <c r="K33" s="190" t="inlineStr">
         <is>
           <t>Arm-dominant paddling · Rapid volume increase · Neglecting shoulder antagonist work · Insufficient core/balance base</t>
         </is>
       </c>
-      <c r="L33" t="inlineStr">
+      <c r="L33" s="190" t="inlineStr">
         <is>
           <t>Same as Kayaking (D-010): rotator-cuff external rotation, wrist extensor stretch, hip flexor stretch.</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr">
+      <c r="M33" s="190" t="inlineStr">
         <is>
           <t>SUP-specific: extrapolated from kayak/canoe paddle-sports literature (Moderate).</t>
         </is>
@@ -15154,8 +15154,8 @@
   <mergeCells count="16">
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="B7:F7"/>
     <mergeCell ref="C31:F31"/>
-    <mergeCell ref="B7:F7"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="C35:F35"/>
     <mergeCell ref="A1:F1"/>

</xml_diff>